<commit_message>
Mise à jour valuebets 2025-07-07 21:04:09
</commit_message>
<xml_diff>
--- a/data/valuebets_database_2025-07-07.xlsx
+++ b/data/valuebets_database_2025-07-07.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H23"/>
+  <dimension ref="A1:H24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -476,7 +476,7 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>45845.8754159185</v>
+        <v>45845.87541591435</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
@@ -498,10 +498,8 @@
           <t>11/07 21:30</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>55.00</t>
-        </is>
+      <c r="F2" t="n">
+        <v>55</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
@@ -516,7 +514,7 @@
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
-        <v>45845.8754159185</v>
+        <v>45845.87541591435</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
@@ -538,10 +536,8 @@
           <t>12/07 21:00</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>45.00</t>
-        </is>
+      <c r="F3" t="n">
+        <v>45</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
@@ -556,7 +552,7 @@
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
-        <v>45845.8754159185</v>
+        <v>45845.87541591435</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
@@ -578,10 +574,8 @@
           <t>12/07 15:30</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>60.00</t>
-        </is>
+      <c r="F4" t="n">
+        <v>60</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
@@ -596,7 +590,7 @@
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
-        <v>45845.8754159185</v>
+        <v>45845.87541591435</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
@@ -618,10 +612,8 @@
           <t>12/07 14:00</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>60.00</t>
-        </is>
+      <c r="F5" t="n">
+        <v>60</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
@@ -636,7 +628,7 @@
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
-        <v>45845.8754159185</v>
+        <v>45845.87541591435</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
@@ -658,10 +650,8 @@
           <t>13/07 14:30</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>60.00</t>
-        </is>
+      <c r="F6" t="n">
+        <v>60</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
@@ -676,7 +666,7 @@
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
-        <v>45845.8754159185</v>
+        <v>45845.87541591435</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
@@ -698,10 +688,8 @@
           <t>08/07 19:00</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>3.00</t>
-        </is>
+      <c r="F7" t="n">
+        <v>3</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
@@ -716,7 +704,7 @@
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
-        <v>45845.8754159185</v>
+        <v>45845.87541591435</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
@@ -738,10 +726,8 @@
           <t>09/07 19:00</t>
         </is>
       </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>3.30</t>
-        </is>
+      <c r="F8" t="n">
+        <v>3.3</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
@@ -756,7 +742,7 @@
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
-        <v>45845.8754159185</v>
+        <v>45845.87541591435</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
@@ -778,10 +764,8 @@
           <t>08/07 13:40</t>
         </is>
       </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>55.00</t>
-        </is>
+      <c r="F9" t="n">
+        <v>55</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>
@@ -796,7 +780,7 @@
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
-        <v>45845.8754159185</v>
+        <v>45845.87541591435</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
@@ -818,10 +802,8 @@
           <t>08/07 16:00</t>
         </is>
       </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>45.00</t>
-        </is>
+      <c r="F10" t="n">
+        <v>45</v>
       </c>
       <c r="G10" t="inlineStr">
         <is>
@@ -836,7 +818,7 @@
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
-        <v>45845.8754159185</v>
+        <v>45845.87541591435</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
@@ -858,10 +840,8 @@
           <t>12/07 19:00</t>
         </is>
       </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>45.00</t>
-        </is>
+      <c r="F11" t="n">
+        <v>45</v>
       </c>
       <c r="G11" t="inlineStr">
         <is>
@@ -876,7 +856,7 @@
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
-        <v>45845.8754159185</v>
+        <v>45845.87541591435</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
@@ -898,10 +878,8 @@
           <t>07/07 23:30</t>
         </is>
       </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>20.00</t>
-        </is>
+      <c r="F12" t="n">
+        <v>20</v>
       </c>
       <c r="G12" t="inlineStr">
         <is>
@@ -916,7 +894,7 @@
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
-        <v>45845.8754159185</v>
+        <v>45845.87541591435</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
@@ -938,10 +916,8 @@
           <t>08/07 15:30</t>
         </is>
       </c>
-      <c r="F13" t="inlineStr">
-        <is>
-          <t>40.00</t>
-        </is>
+      <c r="F13" t="n">
+        <v>40</v>
       </c>
       <c r="G13" t="inlineStr">
         <is>
@@ -956,7 +932,7 @@
     </row>
     <row r="14">
       <c r="A14" s="2" t="n">
-        <v>45845.8754159185</v>
+        <v>45845.87541591435</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
@@ -978,10 +954,8 @@
           <t>08/07 17:00</t>
         </is>
       </c>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t>45.00</t>
-        </is>
+      <c r="F14" t="n">
+        <v>45</v>
       </c>
       <c r="G14" t="inlineStr">
         <is>
@@ -996,7 +970,7 @@
     </row>
     <row r="15">
       <c r="A15" s="2" t="n">
-        <v>45845.8754159185</v>
+        <v>45845.87541591435</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
@@ -1018,10 +992,8 @@
           <t>08/07 16:30</t>
         </is>
       </c>
-      <c r="F15" t="inlineStr">
-        <is>
-          <t>1.32</t>
-        </is>
+      <c r="F15" t="n">
+        <v>1.32</v>
       </c>
       <c r="G15" t="inlineStr">
         <is>
@@ -1036,7 +1008,7 @@
     </row>
     <row r="16">
       <c r="A16" s="2" t="n">
-        <v>45845.8754159185</v>
+        <v>45845.87541591435</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
@@ -1058,10 +1030,8 @@
           <t>08/07 19:00</t>
         </is>
       </c>
-      <c r="F16" t="inlineStr">
-        <is>
-          <t>1.04</t>
-        </is>
+      <c r="F16" t="n">
+        <v>1.04</v>
       </c>
       <c r="G16" t="inlineStr">
         <is>
@@ -1076,7 +1046,7 @@
     </row>
     <row r="17">
       <c r="A17" s="2" t="n">
-        <v>45845.8754159185</v>
+        <v>45845.87541591435</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
@@ -1098,10 +1068,8 @@
           <t>08/07 16:00</t>
         </is>
       </c>
-      <c r="F17" t="inlineStr">
-        <is>
-          <t>1.11</t>
-        </is>
+      <c r="F17" t="n">
+        <v>1.11</v>
       </c>
       <c r="G17" t="inlineStr">
         <is>
@@ -1116,7 +1084,7 @@
     </row>
     <row r="18">
       <c r="A18" s="2" t="n">
-        <v>45845.8754159185</v>
+        <v>45845.87541591435</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
@@ -1138,10 +1106,8 @@
           <t>09/07 17:30</t>
         </is>
       </c>
-      <c r="F18" t="inlineStr">
-        <is>
-          <t>1.10</t>
-        </is>
+      <c r="F18" t="n">
+        <v>1.1</v>
       </c>
       <c r="G18" t="inlineStr">
         <is>
@@ -1156,7 +1122,7 @@
     </row>
     <row r="19">
       <c r="A19" s="2" t="n">
-        <v>45845.8754159185</v>
+        <v>45845.87541591435</v>
       </c>
       <c r="B19" t="inlineStr">
         <is>
@@ -1178,10 +1144,8 @@
           <t>08/07 15:00</t>
         </is>
       </c>
-      <c r="F19" t="inlineStr">
-        <is>
-          <t>1.11</t>
-        </is>
+      <c r="F19" t="n">
+        <v>1.11</v>
       </c>
       <c r="G19" t="inlineStr">
         <is>
@@ -1196,7 +1160,7 @@
     </row>
     <row r="20">
       <c r="A20" s="2" t="n">
-        <v>45845.8754159185</v>
+        <v>45845.87541591435</v>
       </c>
       <c r="B20" t="inlineStr">
         <is>
@@ -1218,10 +1182,8 @@
           <t>08/07 18:00</t>
         </is>
       </c>
-      <c r="F20" t="inlineStr">
-        <is>
-          <t>1.24</t>
-        </is>
+      <c r="F20" t="n">
+        <v>1.24</v>
       </c>
       <c r="G20" t="inlineStr">
         <is>
@@ -1236,7 +1198,7 @@
     </row>
     <row r="21">
       <c r="A21" s="2" t="n">
-        <v>45845.8754159185</v>
+        <v>45845.87541591435</v>
       </c>
       <c r="B21" t="inlineStr">
         <is>
@@ -1258,10 +1220,8 @@
           <t>09/07 17:30</t>
         </is>
       </c>
-      <c r="F21" t="inlineStr">
-        <is>
-          <t>1.04</t>
-        </is>
+      <c r="F21" t="n">
+        <v>1.04</v>
       </c>
       <c r="G21" t="inlineStr">
         <is>
@@ -1276,7 +1236,7 @@
     </row>
     <row r="22">
       <c r="A22" s="2" t="n">
-        <v>45845.8754159185</v>
+        <v>45845.87541591435</v>
       </c>
       <c r="B22" t="inlineStr">
         <is>
@@ -1298,10 +1258,8 @@
           <t>08/07 16:00</t>
         </is>
       </c>
-      <c r="F22" t="inlineStr">
-        <is>
-          <t>1.16</t>
-        </is>
+      <c r="F22" t="n">
+        <v>1.16</v>
       </c>
       <c r="G22" t="inlineStr">
         <is>
@@ -1316,7 +1274,7 @@
     </row>
     <row r="23">
       <c r="A23" s="2" t="n">
-        <v>45845.8754159185</v>
+        <v>45845.87541591435</v>
       </c>
       <c r="B23" t="inlineStr">
         <is>
@@ -1338,10 +1296,8 @@
           <t>08/07 18:00</t>
         </is>
       </c>
-      <c r="F23" t="inlineStr">
-        <is>
-          <t>1.22</t>
-        </is>
+      <c r="F23" t="n">
+        <v>1.22</v>
       </c>
       <c r="G23" t="inlineStr">
         <is>
@@ -1351,6 +1307,46 @@
       <c r="H23" t="inlineStr">
         <is>
           <t>+0,65%</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="n">
+        <v>45845.87779640548</v>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Bwin(FR)Football</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Fotbal Club FCSB – Inter Club d'EscaldesEurope - Ligue des Champions</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>2 / HNB</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>09/07 17:30</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>4.20</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>24,1%</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>+1,07%</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Mise à jour valuebets 2025-07-07 21:21:16
</commit_message>
<xml_diff>
--- a/data/valuebets_database_2025-07-07.xlsx
+++ b/data/valuebets_database_2025-07-07.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H24"/>
+  <dimension ref="A1:H25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1312,7 +1312,7 @@
     </row>
     <row r="24">
       <c r="A24" s="2" t="n">
-        <v>45845.87779640548</v>
+        <v>45845.87779640046</v>
       </c>
       <c r="B24" t="inlineStr">
         <is>
@@ -1334,10 +1334,8 @@
           <t>09/07 17:30</t>
         </is>
       </c>
-      <c r="F24" t="inlineStr">
-        <is>
-          <t>4.20</t>
-        </is>
+      <c r="F24" t="n">
+        <v>4.2</v>
       </c>
       <c r="G24" t="inlineStr">
         <is>
@@ -1347,6 +1345,46 @@
       <c r="H24" t="inlineStr">
         <is>
           <t>+1,07%</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="n">
+        <v>45845.88967684034</v>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Winamax(FR)Football</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>KuPS – FC Milsami OrheiEurope - Ligue des Champions</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>1X</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>08/07 15:00</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>1.11</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>91,1%</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>+1,09%</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Mise à jour valuebets 2025-07-07 22:21:57
</commit_message>
<xml_diff>
--- a/data/valuebets_database_2025-07-07.xlsx
+++ b/data/valuebets_database_2025-07-07.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H25"/>
+  <dimension ref="A1:H27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1350,7 +1350,7 @@
     </row>
     <row r="25">
       <c r="A25" s="2" t="n">
-        <v>45845.88967684034</v>
+        <v>45845.88967684028</v>
       </c>
       <c r="B25" t="inlineStr">
         <is>
@@ -1372,10 +1372,8 @@
           <t>08/07 15:00</t>
         </is>
       </c>
-      <c r="F25" t="inlineStr">
-        <is>
-          <t>1.11</t>
-        </is>
+      <c r="F25" t="n">
+        <v>1.11</v>
       </c>
       <c r="G25" t="inlineStr">
         <is>
@@ -1385,6 +1383,86 @@
       <c r="H25" t="inlineStr">
         <is>
           <t>+1,09%</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="n">
+        <v>45845.9318162729</v>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>BetClic(FR)Football</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Fluminense – ChelseaInternational - Coupe du Monde des Clubs 2025</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Moins que 22.5 - tirs</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>08/07 19:00</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>3.20</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>35,5%</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>+13,7%</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="n">
+        <v>45845.9318162729</v>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Unibet(FR)Football</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Sportivo Ameliano – Cerro PortenoPrimera Division</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Plus que 3.51re équipe</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>12/07 18:30</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>35.00</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>2,88%</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>+0,72%</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Mise à jour valuebets 2025-07-07 23:21:18
</commit_message>
<xml_diff>
--- a/data/valuebets_database_2025-07-07.xlsx
+++ b/data/valuebets_database_2025-07-07.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H27"/>
+  <dimension ref="A1:H29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1388,7 +1388,7 @@
     </row>
     <row r="26">
       <c r="A26" s="2" t="n">
-        <v>45845.9318162729</v>
+        <v>45845.93181627315</v>
       </c>
       <c r="B26" t="inlineStr">
         <is>
@@ -1410,10 +1410,8 @@
           <t>08/07 19:00</t>
         </is>
       </c>
-      <c r="F26" t="inlineStr">
-        <is>
-          <t>3.20</t>
-        </is>
+      <c r="F26" t="n">
+        <v>3.2</v>
       </c>
       <c r="G26" t="inlineStr">
         <is>
@@ -1428,7 +1426,7 @@
     </row>
     <row r="27">
       <c r="A27" s="2" t="n">
-        <v>45845.9318162729</v>
+        <v>45845.93181627315</v>
       </c>
       <c r="B27" t="inlineStr">
         <is>
@@ -1450,10 +1448,8 @@
           <t>12/07 18:30</t>
         </is>
       </c>
-      <c r="F27" t="inlineStr">
-        <is>
-          <t>35.00</t>
-        </is>
+      <c r="F27" t="n">
+        <v>35</v>
       </c>
       <c r="G27" t="inlineStr">
         <is>
@@ -1463,6 +1459,86 @@
       <c r="H27" t="inlineStr">
         <is>
           <t>+0,72%</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="n">
+        <v>45845.97304665373</v>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>BetClic(FR)Football</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Fluminense – ChelseaInternational - Coupe du Monde des Clubs 2025 A9ZJ2X7R 385076e7</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Moins que 22.5 - tirs</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>08/07 19:00</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>2.95</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>37,1%</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>+9,34%</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="n">
+        <v>45845.97304665373</v>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>BetClic(FR)Football</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>KF Drita – Differdange 03Europe - Ligue des Champions</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>11-2- se qualifie</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>08/07 18:00</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>1.65</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>61,5%</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>+1,54%</t>
         </is>
       </c>
     </row>

</xml_diff>